<commit_message>
[Firmware] Chore: hago commit con tareas intermedias para salvar el trabajo y hacer pruebas en otras ramas.
</commit_message>
<xml_diff>
--- a/Administracion/08 - Logger consumo y capacidad.xlsx
+++ b/Administracion/08 - Logger consumo y capacidad.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28827"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\FLOWMEET Dropbox\flowmeet\ID\Electronica\Equipos\FMC-320U\Administracion\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\githubs\FMC-320U\Administracion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D98EE65-C09D-4A8C-BBFD-5F5AC13BCBEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD1C982E-51E1-40D3-90D8-33298BB64C22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Leer" sheetId="5" r:id="rId1"/>
@@ -147,7 +147,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="68">
   <si>
     <t>Memoria Inicial</t>
   </si>
@@ -353,16 +353,22 @@
     <t>Impresiones por dia</t>
   </si>
   <si>
-    <t>Impresiones en  5 años</t>
-  </si>
-  <si>
     <t>Impresión soportadas para uso del 15% de la bateria</t>
   </si>
   <si>
-    <t>Reservo el 15% de la capacidad de la bateria para descarga de datos o imprimir ticket. Con esto puede descargar datos mas de una vez a la semana o imprimir dos tickets por dia.</t>
-  </si>
-  <si>
     <t>Nota, las mediciones en este caso se hicieron con el ST-LKINK desconectado, si se conecta el ST-LINK hay un drenaje de corriente desde ST-LINK hacia el computador, y el consumo disminuye 5uA aproximadamente.</t>
+  </si>
+  <si>
+    <t>Reservo el 15% de la capacidad de la bateria para descarga de datos o imprimir ticket.</t>
+  </si>
+  <si>
+    <t>Años de autonnomia</t>
+  </si>
+  <si>
+    <t>Suponiendo que el equipo funciona 8 horas al día, los 365 días del año, y asignando un 15% de la capacidad de la batería al data logger o a la impresión de tickets:
+En el caso de imprimir 3 tickets por dia, 365 dias al año, la vida útil estimada de la batería sería superior a 4,09 años.
+Si se descargan los datos una vez por semana, con una conexión de 120 segundos, la vida útil estimada de la batería sería superior a 4,32 años.
+Ambos escenarios son muy desfavorables. Por lo tanto, es razonable establecer una vida útil nominal de 5 años para la batería.</t>
   </si>
 </sst>
 </file>
@@ -372,7 +378,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -434,6 +440,12 @@
       <name val="Tahoma"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -637,7 +649,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -652,9 +664,14 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="1" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -709,76 +726,59 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="1" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -796,10 +796,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1069,56 +1065,56 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="3" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B3" s="35" t="s">
-        <v>66</v>
-      </c>
-      <c r="C3" s="53"/>
-      <c r="D3" s="53"/>
-      <c r="E3" s="53"/>
-      <c r="F3" s="53"/>
-      <c r="G3" s="53"/>
-      <c r="H3" s="53"/>
-      <c r="I3" s="53"/>
+      <c r="B3" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="C3" s="11"/>
+      <c r="D3" s="11"/>
+      <c r="E3" s="11"/>
+      <c r="F3" s="11"/>
+      <c r="G3" s="11"/>
+      <c r="H3" s="11"/>
+      <c r="I3" s="11"/>
     </row>
     <row r="4" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B4" s="53"/>
-      <c r="C4" s="53"/>
-      <c r="D4" s="53"/>
-      <c r="E4" s="53"/>
-      <c r="F4" s="53"/>
-      <c r="G4" s="53"/>
-      <c r="H4" s="53"/>
-      <c r="I4" s="53"/>
+      <c r="B4" s="11"/>
+      <c r="C4" s="11"/>
+      <c r="D4" s="11"/>
+      <c r="E4" s="11"/>
+      <c r="F4" s="11"/>
+      <c r="G4" s="11"/>
+      <c r="H4" s="11"/>
+      <c r="I4" s="11"/>
     </row>
     <row r="5" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B5" s="53"/>
-      <c r="C5" s="53"/>
-      <c r="D5" s="53"/>
-      <c r="E5" s="53"/>
-      <c r="F5" s="53"/>
-      <c r="G5" s="53"/>
-      <c r="H5" s="53"/>
-      <c r="I5" s="53"/>
+      <c r="B5" s="11"/>
+      <c r="C5" s="11"/>
+      <c r="D5" s="11"/>
+      <c r="E5" s="11"/>
+      <c r="F5" s="11"/>
+      <c r="G5" s="11"/>
+      <c r="H5" s="11"/>
+      <c r="I5" s="11"/>
     </row>
     <row r="6" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B6" s="53"/>
-      <c r="C6" s="53"/>
-      <c r="D6" s="53"/>
-      <c r="E6" s="53"/>
-      <c r="F6" s="53"/>
-      <c r="G6" s="53"/>
-      <c r="H6" s="53"/>
-      <c r="I6" s="53"/>
+      <c r="B6" s="11"/>
+      <c r="C6" s="11"/>
+      <c r="D6" s="11"/>
+      <c r="E6" s="11"/>
+      <c r="F6" s="11"/>
+      <c r="G6" s="11"/>
+      <c r="H6" s="11"/>
+      <c r="I6" s="11"/>
     </row>
     <row r="7" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B7" s="53"/>
-      <c r="C7" s="53"/>
-      <c r="D7" s="53"/>
-      <c r="E7" s="53"/>
-      <c r="F7" s="53"/>
-      <c r="G7" s="53"/>
-      <c r="H7" s="53"/>
-      <c r="I7" s="53"/>
+      <c r="B7" s="11"/>
+      <c r="C7" s="11"/>
+      <c r="D7" s="11"/>
+      <c r="E7" s="11"/>
+      <c r="F7" s="11"/>
+      <c r="G7" s="11"/>
+      <c r="H7" s="11"/>
+      <c r="I7" s="11"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1482,11 +1478,11 @@
         <f t="shared" ref="G5:G6" si="0">F5</f>
         <v>450</v>
       </c>
-      <c r="H5" s="9">
+      <c r="H5" s="46">
         <f t="shared" ref="H5:H6" si="1">F5*7</f>
         <v>3150</v>
       </c>
-      <c r="I5" s="8">
+      <c r="I5" s="47">
         <f t="shared" ref="I5:I6" si="2">H5/365</f>
         <v>8.6301369863013697</v>
       </c>
@@ -1506,7 +1502,7 @@
       <c r="C6" s="4">
         <v>70</v>
       </c>
-      <c r="D6" s="4">
+      <c r="D6" s="48">
         <f>D5*2</f>
         <v>120</v>
       </c>
@@ -1523,11 +1519,11 @@
         <v>225</v>
       </c>
       <c r="H6" s="4">
-        <f t="shared" si="1"/>
+        <f>F6*7</f>
         <v>1575</v>
       </c>
       <c r="I6" s="7">
-        <f t="shared" si="2"/>
+        <f>H6/365</f>
         <v>4.3150684931506849</v>
       </c>
       <c r="J6" s="5">
@@ -1540,105 +1536,105 @@
       </c>
     </row>
     <row r="9" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="20" t="s">
+      <c r="B9" s="21" t="s">
         <v>27</v>
       </c>
-      <c r="C9" s="21"/>
-      <c r="D9" s="21"/>
-      <c r="E9" s="21"/>
-      <c r="F9" s="21"/>
-      <c r="G9" s="22"/>
+      <c r="C9" s="22"/>
+      <c r="D9" s="22"/>
+      <c r="E9" s="22"/>
+      <c r="F9" s="22"/>
+      <c r="G9" s="23"/>
       <c r="H9" s="6"/>
       <c r="I9" s="6"/>
       <c r="J9" s="6"/>
       <c r="K9" s="6"/>
     </row>
     <row r="10" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B10" s="23"/>
-      <c r="C10" s="24"/>
-      <c r="D10" s="24"/>
-      <c r="E10" s="24"/>
-      <c r="F10" s="24"/>
-      <c r="G10" s="25"/>
+      <c r="B10" s="24"/>
+      <c r="C10" s="25"/>
+      <c r="D10" s="25"/>
+      <c r="E10" s="25"/>
+      <c r="F10" s="25"/>
+      <c r="G10" s="26"/>
       <c r="H10" s="6"/>
       <c r="I10" s="6"/>
       <c r="J10" s="6"/>
       <c r="K10" s="6"/>
     </row>
     <row r="11" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B11" s="23"/>
-      <c r="C11" s="24"/>
-      <c r="D11" s="24"/>
-      <c r="E11" s="24"/>
-      <c r="F11" s="24"/>
-      <c r="G11" s="25"/>
+      <c r="B11" s="24"/>
+      <c r="C11" s="25"/>
+      <c r="D11" s="25"/>
+      <c r="E11" s="25"/>
+      <c r="F11" s="25"/>
+      <c r="G11" s="26"/>
       <c r="H11" s="6"/>
       <c r="I11" s="6"/>
       <c r="J11" s="6"/>
       <c r="K11" s="6"/>
     </row>
     <row r="12" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B12" s="23"/>
-      <c r="C12" s="24"/>
-      <c r="D12" s="24"/>
-      <c r="E12" s="24"/>
-      <c r="F12" s="24"/>
-      <c r="G12" s="25"/>
+      <c r="B12" s="24"/>
+      <c r="C12" s="25"/>
+      <c r="D12" s="25"/>
+      <c r="E12" s="25"/>
+      <c r="F12" s="25"/>
+      <c r="G12" s="26"/>
       <c r="H12" s="6"/>
       <c r="I12" s="6"/>
       <c r="J12" s="6"/>
       <c r="K12" s="6"/>
     </row>
     <row r="13" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B13" s="23" t="s">
+      <c r="B13" s="24" t="s">
         <v>28</v>
       </c>
-      <c r="C13" s="24"/>
-      <c r="D13" s="24"/>
-      <c r="E13" s="24"/>
-      <c r="F13" s="24"/>
-      <c r="G13" s="25"/>
+      <c r="C13" s="25"/>
+      <c r="D13" s="25"/>
+      <c r="E13" s="25"/>
+      <c r="F13" s="25"/>
+      <c r="G13" s="26"/>
       <c r="H13" s="6"/>
       <c r="I13" s="6"/>
       <c r="J13" s="6"/>
       <c r="K13" s="6"/>
     </row>
     <row r="14" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B14" s="26" t="s">
+      <c r="B14" s="27" t="s">
         <v>29</v>
       </c>
-      <c r="C14" s="27"/>
-      <c r="D14" s="27"/>
-      <c r="E14" s="27"/>
-      <c r="F14" s="27"/>
-      <c r="G14" s="28"/>
+      <c r="C14" s="28"/>
+      <c r="D14" s="28"/>
+      <c r="E14" s="28"/>
+      <c r="F14" s="28"/>
+      <c r="G14" s="29"/>
       <c r="H14" s="6"/>
       <c r="I14" s="6"/>
       <c r="J14" s="6"/>
       <c r="K14" s="6"/>
     </row>
     <row r="16" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B16" s="11" t="s">
+      <c r="B16" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="C16" s="12"/>
-      <c r="D16" s="12"/>
-      <c r="E16" s="12"/>
-      <c r="F16" s="13"/>
+      <c r="C16" s="13"/>
+      <c r="D16" s="13"/>
+      <c r="E16" s="13"/>
+      <c r="F16" s="14"/>
     </row>
     <row r="17" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B17" s="14"/>
-      <c r="C17" s="15"/>
-      <c r="D17" s="15"/>
-      <c r="E17" s="15"/>
-      <c r="F17" s="16"/>
+      <c r="B17" s="15"/>
+      <c r="C17" s="16"/>
+      <c r="D17" s="16"/>
+      <c r="E17" s="16"/>
+      <c r="F17" s="17"/>
     </row>
     <row r="18" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B18" s="17"/>
-      <c r="C18" s="18"/>
-      <c r="D18" s="18"/>
-      <c r="E18" s="18"/>
-      <c r="F18" s="19"/>
+      <c r="B18" s="18"/>
+      <c r="C18" s="19"/>
+      <c r="D18" s="19"/>
+      <c r="E18" s="19"/>
+      <c r="F18" s="20"/>
     </row>
     <row r="20" spans="2:11" ht="75" x14ac:dyDescent="0.25">
       <c r="B20" s="3" t="s">
@@ -1738,7 +1734,7 @@
         <f t="shared" ref="H22:H23" si="5">F22*7</f>
         <v>7350</v>
       </c>
-      <c r="I22" s="10">
+      <c r="I22" s="8">
         <f t="shared" ref="I22:I23" si="6">H22/365</f>
         <v>20.136986301369863</v>
       </c>
@@ -1792,27 +1788,27 @@
       </c>
     </row>
     <row r="25" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B25" s="11" t="s">
+      <c r="B25" s="12" t="s">
         <v>31</v>
       </c>
-      <c r="C25" s="12"/>
-      <c r="D25" s="12"/>
-      <c r="E25" s="12"/>
-      <c r="F25" s="13"/>
+      <c r="C25" s="13"/>
+      <c r="D25" s="13"/>
+      <c r="E25" s="13"/>
+      <c r="F25" s="14"/>
     </row>
     <row r="26" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B26" s="14"/>
-      <c r="C26" s="15"/>
-      <c r="D26" s="15"/>
-      <c r="E26" s="15"/>
-      <c r="F26" s="16"/>
+      <c r="B26" s="15"/>
+      <c r="C26" s="16"/>
+      <c r="D26" s="16"/>
+      <c r="E26" s="16"/>
+      <c r="F26" s="17"/>
     </row>
     <row r="27" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B27" s="17"/>
-      <c r="C27" s="18"/>
-      <c r="D27" s="18"/>
-      <c r="E27" s="18"/>
-      <c r="F27" s="19"/>
+      <c r="B27" s="18"/>
+      <c r="C27" s="19"/>
+      <c r="D27" s="19"/>
+      <c r="E27" s="19"/>
+      <c r="F27" s="20"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -1835,32 +1831,30 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B2" s="37" t="s">
+      <c r="B2" s="30" t="s">
         <v>56</v>
       </c>
-      <c r="C2" s="37"/>
-      <c r="D2" s="37"/>
-      <c r="E2" s="37"/>
-      <c r="F2" s="37"/>
-      <c r="G2" s="37"/>
+      <c r="C2" s="30"/>
+      <c r="D2" s="30"/>
+      <c r="E2" s="30"/>
+      <c r="F2" s="30"/>
+      <c r="G2" s="30"/>
     </row>
     <row r="3" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B3" s="37"/>
-      <c r="C3" s="37"/>
-      <c r="D3" s="37"/>
-      <c r="E3" s="37"/>
-      <c r="F3" s="37"/>
-      <c r="G3" s="37"/>
+      <c r="B3" s="30"/>
+      <c r="C3" s="30"/>
+      <c r="D3" s="30"/>
+      <c r="E3" s="30"/>
+      <c r="F3" s="30"/>
+      <c r="G3" s="30"/>
     </row>
     <row r="5" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B5" s="29" t="s">
+      <c r="B5" s="31" t="s">
         <v>57</v>
       </c>
-      <c r="C5" s="29"/>
-      <c r="D5" s="29"/>
-      <c r="E5" s="29"/>
-      <c r="F5" s="52"/>
-      <c r="G5" s="52"/>
+      <c r="C5" s="31"/>
+      <c r="D5" s="31"/>
+      <c r="E5" s="31"/>
     </row>
     <row r="6" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
@@ -1895,13 +1889,13 @@
         <v>61</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="F10" s="3" t="s">
         <v>62</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
     </row>
     <row r="11" spans="2:7" x14ac:dyDescent="0.25">
@@ -1921,9 +1915,9 @@
       <c r="F11" s="5">
         <v>1</v>
       </c>
-      <c r="G11" s="5">
-        <f>F11*365*5</f>
-        <v>1825</v>
+      <c r="G11" s="7">
+        <f>E11/(365*F11)</f>
+        <v>12.281978633256216</v>
       </c>
     </row>
     <row r="12" spans="2:7" x14ac:dyDescent="0.25">
@@ -1943,9 +1937,9 @@
       <c r="F12" s="5">
         <v>2</v>
       </c>
-      <c r="G12" s="5">
-        <f t="shared" ref="G12:G13" si="1">F12*365*5</f>
-        <v>3650</v>
+      <c r="G12" s="7">
+        <f t="shared" ref="G12:G13" si="1">E12/(365*F12)</f>
+        <v>6.140989316628108</v>
       </c>
     </row>
     <row r="13" spans="2:7" x14ac:dyDescent="0.25">
@@ -1963,11 +1957,11 @@
         <v>4482.9222011385191</v>
       </c>
       <c r="F13" s="5">
-        <v>5</v>
-      </c>
-      <c r="G13" s="5">
+        <v>3</v>
+      </c>
+      <c r="G13" s="7">
         <f t="shared" si="1"/>
-        <v>9125</v>
+        <v>4.093992877752072</v>
       </c>
     </row>
   </sheetData>
@@ -1981,7 +1975,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{05F4793D-FBB7-40C9-B5F6-023AD69CC458}">
-  <dimension ref="B2:O20"/>
+  <dimension ref="B2:S20"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="3" customWidth="1"/>
@@ -1994,56 +1988,56 @@
     <col min="15" max="15" width="14.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="11" t="s">
+    <row r="2" spans="2:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2" s="12" t="s">
         <v>45</v>
       </c>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12"/>
-      <c r="E2" s="12"/>
-      <c r="F2" s="12"/>
-      <c r="G2" s="12"/>
-      <c r="H2" s="12"/>
-      <c r="I2" s="12"/>
-      <c r="J2" s="12"/>
-      <c r="K2" s="12"/>
-      <c r="L2" s="12"/>
-      <c r="M2" s="12"/>
-      <c r="N2" s="12"/>
-      <c r="O2" s="13"/>
-    </row>
-    <row r="3" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B3" s="17"/>
-      <c r="C3" s="18"/>
-      <c r="D3" s="18"/>
-      <c r="E3" s="18"/>
-      <c r="F3" s="18"/>
-      <c r="G3" s="18"/>
-      <c r="H3" s="18"/>
-      <c r="I3" s="18"/>
-      <c r="J3" s="18"/>
-      <c r="K3" s="18"/>
-      <c r="L3" s="18"/>
-      <c r="M3" s="18"/>
-      <c r="N3" s="18"/>
-      <c r="O3" s="19"/>
-    </row>
-    <row r="4" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B4" s="38"/>
-      <c r="C4" s="38"/>
-      <c r="D4" s="38"/>
-      <c r="E4" s="38"/>
-      <c r="F4" s="38"/>
-      <c r="G4" s="38"/>
-      <c r="H4" s="38"/>
-      <c r="I4" s="38"/>
-      <c r="J4" s="38"/>
-      <c r="K4" s="38"/>
-      <c r="L4" s="38"/>
-      <c r="M4" s="38"/>
-      <c r="N4" s="38"/>
-    </row>
-    <row r="5" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="C2" s="13"/>
+      <c r="D2" s="13"/>
+      <c r="E2" s="13"/>
+      <c r="F2" s="13"/>
+      <c r="G2" s="13"/>
+      <c r="H2" s="13"/>
+      <c r="I2" s="13"/>
+      <c r="J2" s="13"/>
+      <c r="K2" s="13"/>
+      <c r="L2" s="13"/>
+      <c r="M2" s="13"/>
+      <c r="N2" s="13"/>
+      <c r="O2" s="14"/>
+    </row>
+    <row r="3" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B3" s="18"/>
+      <c r="C3" s="19"/>
+      <c r="D3" s="19"/>
+      <c r="E3" s="19"/>
+      <c r="F3" s="19"/>
+      <c r="G3" s="19"/>
+      <c r="H3" s="19"/>
+      <c r="I3" s="19"/>
+      <c r="J3" s="19"/>
+      <c r="K3" s="19"/>
+      <c r="L3" s="19"/>
+      <c r="M3" s="19"/>
+      <c r="N3" s="19"/>
+      <c r="O3" s="20"/>
+    </row>
+    <row r="4" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B4" s="6"/>
+      <c r="C4" s="6"/>
+      <c r="D4" s="6"/>
+      <c r="E4" s="6"/>
+      <c r="F4" s="6"/>
+      <c r="G4" s="6"/>
+      <c r="H4" s="6"/>
+      <c r="I4" s="6"/>
+      <c r="J4" s="6"/>
+      <c r="K4" s="6"/>
+      <c r="L4" s="6"/>
+      <c r="M4" s="6"/>
+      <c r="N4" s="6"/>
+    </row>
+    <row r="5" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B5" s="4" t="s">
         <v>33</v>
       </c>
@@ -2059,41 +2053,41 @@
       <c r="F5" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="H5" s="30" t="s">
+      <c r="H5" s="38" t="s">
         <v>46</v>
       </c>
-      <c r="I5" s="30"/>
-      <c r="J5" s="30"/>
-      <c r="K5" s="30"/>
-      <c r="L5" s="30"/>
-      <c r="M5" s="30"/>
-      <c r="N5" s="30"/>
-      <c r="O5" s="30"/>
-    </row>
-    <row r="6" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="I5" s="38"/>
+      <c r="J5" s="38"/>
+      <c r="K5" s="38"/>
+      <c r="L5" s="38"/>
+      <c r="M5" s="38"/>
+      <c r="N5" s="38"/>
+      <c r="O5" s="38"/>
+    </row>
+    <row r="6" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B6" s="4" t="s">
         <v>36</v>
       </c>
       <c r="C6" s="4">
         <v>40</v>
       </c>
-      <c r="D6" s="31">
+      <c r="D6" s="9">
         <f>2/3</f>
         <v>0.66666666666666663</v>
       </c>
-      <c r="E6" s="10">
+      <c r="E6" s="8">
         <f>C6*D6</f>
         <v>26.666666666666664</v>
       </c>
       <c r="F6" s="4"/>
-      <c r="H6" s="30" t="s">
+      <c r="H6" s="38" t="s">
         <v>35</v>
       </c>
-      <c r="I6" s="30"/>
-      <c r="J6" s="34" t="s">
+      <c r="I6" s="38"/>
+      <c r="J6" s="45" t="s">
         <v>48</v>
       </c>
-      <c r="K6" s="34"/>
+      <c r="K6" s="45"/>
       <c r="L6" s="4" t="s">
         <v>50</v>
       </c>
@@ -2107,30 +2101,30 @@
         <v>55</v>
       </c>
     </row>
-    <row r="7" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B7" s="4" t="s">
         <v>38</v>
       </c>
       <c r="C7" s="4">
         <v>78</v>
       </c>
-      <c r="D7" s="31">
+      <c r="D7" s="9">
         <f>1/3</f>
         <v>0.33333333333333331</v>
       </c>
-      <c r="E7" s="10">
+      <c r="E7" s="8">
         <f>C7*D7</f>
         <v>26</v>
       </c>
       <c r="F7" s="4"/>
-      <c r="H7" s="30" t="s">
+      <c r="H7" s="38" t="s">
         <v>47</v>
       </c>
-      <c r="I7" s="30"/>
-      <c r="J7" s="30">
+      <c r="I7" s="38"/>
+      <c r="J7" s="38">
         <v>3500</v>
       </c>
-      <c r="K7" s="30"/>
+      <c r="K7" s="38"/>
       <c r="L7" s="4">
         <v>1.7</v>
       </c>
@@ -2145,44 +2139,44 @@
         <v>25</v>
       </c>
     </row>
-    <row r="8" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B8" s="4"/>
       <c r="C8" s="4"/>
       <c r="D8" s="4"/>
       <c r="E8" s="4"/>
       <c r="F8" s="4"/>
-      <c r="H8" s="30"/>
-      <c r="I8" s="30"/>
-      <c r="J8" s="30"/>
-      <c r="K8" s="30"/>
+      <c r="H8" s="38"/>
+      <c r="I8" s="38"/>
+      <c r="J8" s="38"/>
+      <c r="K8" s="38"/>
       <c r="L8" s="4"/>
       <c r="M8" s="4"/>
       <c r="N8" s="4"/>
       <c r="O8" s="4"/>
     </row>
-    <row r="9" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B9" s="4"/>
       <c r="C9" s="4"/>
       <c r="D9" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="E9" s="10">
+      <c r="E9" s="8">
         <f>SUM(E6:E8)</f>
         <v>52.666666666666664</v>
       </c>
       <c r="F9" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="H9" s="30"/>
-      <c r="I9" s="30"/>
-      <c r="J9" s="30"/>
-      <c r="K9" s="30"/>
+      <c r="H9" s="38"/>
+      <c r="I9" s="38"/>
+      <c r="J9" s="38"/>
+      <c r="K9" s="38"/>
       <c r="L9" s="4"/>
       <c r="M9" s="4"/>
       <c r="N9" s="4"/>
       <c r="O9" s="4"/>
     </row>
-    <row r="10" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B10" s="4"/>
       <c r="C10" s="4"/>
       <c r="D10" s="4" t="s">
@@ -2196,13 +2190,13 @@
         <v>43</v>
       </c>
     </row>
-    <row r="11" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B11" s="49" t="s">
+    <row r="11" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B11" s="39" t="s">
         <v>54</v>
       </c>
-      <c r="C11" s="50"/>
-      <c r="D11" s="51"/>
-      <c r="E11" s="10">
+      <c r="C11" s="40"/>
+      <c r="D11" s="41"/>
+      <c r="E11" s="8">
         <f>E10/(24*365)</f>
         <v>6.4483266863187101</v>
       </c>
@@ -2210,87 +2204,196 @@
         <v>44</v>
       </c>
     </row>
-    <row r="12" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B12" s="11" t="s">
+    <row r="12" spans="2:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B12" s="12" t="s">
         <v>65</v>
       </c>
-      <c r="C12" s="12"/>
-      <c r="D12" s="13"/>
-      <c r="E12" s="46">
+      <c r="C12" s="13"/>
+      <c r="D12" s="14"/>
+      <c r="E12" s="32">
         <f>E10*0.85/(365*24)</f>
         <v>5.4810776833709038</v>
       </c>
-      <c r="F12" s="43" t="s">
+      <c r="F12" s="35" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="13" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B13" s="14"/>
-      <c r="C13" s="36"/>
-      <c r="D13" s="16"/>
-      <c r="E13" s="47"/>
-      <c r="F13" s="44"/>
-    </row>
-    <row r="14" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B14" s="14"/>
-      <c r="C14" s="36"/>
-      <c r="D14" s="16"/>
-      <c r="E14" s="47"/>
-      <c r="F14" s="44"/>
-    </row>
-    <row r="15" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="17"/>
-      <c r="C15" s="18"/>
-      <c r="D15" s="19"/>
-      <c r="E15" s="48"/>
-      <c r="F15" s="45"/>
-      <c r="H15" s="40"/>
-      <c r="I15" s="41"/>
-      <c r="J15" s="42"/>
-    </row>
-    <row r="16" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B16" s="32"/>
-      <c r="C16" s="39"/>
-      <c r="D16" s="33"/>
+      <c r="H12" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="I12" s="13"/>
+      <c r="J12" s="13"/>
+      <c r="K12" s="13"/>
+      <c r="L12" s="13"/>
+      <c r="M12" s="13"/>
+      <c r="N12" s="13"/>
+      <c r="O12" s="13"/>
+      <c r="P12" s="13"/>
+      <c r="Q12" s="13"/>
+      <c r="R12" s="13"/>
+      <c r="S12" s="14"/>
+    </row>
+    <row r="13" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B13" s="15"/>
+      <c r="C13" s="16"/>
+      <c r="D13" s="17"/>
+      <c r="E13" s="33"/>
+      <c r="F13" s="36"/>
+      <c r="H13" s="15"/>
+      <c r="I13" s="49"/>
+      <c r="J13" s="49"/>
+      <c r="K13" s="49"/>
+      <c r="L13" s="49"/>
+      <c r="M13" s="49"/>
+      <c r="N13" s="49"/>
+      <c r="O13" s="49"/>
+      <c r="P13" s="49"/>
+      <c r="Q13" s="49"/>
+      <c r="R13" s="49"/>
+      <c r="S13" s="17"/>
+    </row>
+    <row r="14" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B14" s="15"/>
+      <c r="C14" s="16"/>
+      <c r="D14" s="17"/>
+      <c r="E14" s="33"/>
+      <c r="F14" s="36"/>
+      <c r="H14" s="15"/>
+      <c r="I14" s="49"/>
+      <c r="J14" s="49"/>
+      <c r="K14" s="49"/>
+      <c r="L14" s="49"/>
+      <c r="M14" s="49"/>
+      <c r="N14" s="49"/>
+      <c r="O14" s="49"/>
+      <c r="P14" s="49"/>
+      <c r="Q14" s="49"/>
+      <c r="R14" s="49"/>
+      <c r="S14" s="17"/>
+    </row>
+    <row r="15" spans="2:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B15" s="18"/>
+      <c r="C15" s="19"/>
+      <c r="D15" s="20"/>
+      <c r="E15" s="34"/>
+      <c r="F15" s="37"/>
+      <c r="H15" s="15"/>
+      <c r="I15" s="49"/>
+      <c r="J15" s="49"/>
+      <c r="K15" s="49"/>
+      <c r="L15" s="49"/>
+      <c r="M15" s="49"/>
+      <c r="N15" s="49"/>
+      <c r="O15" s="49"/>
+      <c r="P15" s="49"/>
+      <c r="Q15" s="49"/>
+      <c r="R15" s="49"/>
+      <c r="S15" s="17"/>
+    </row>
+    <row r="16" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B16" s="42"/>
+      <c r="C16" s="43"/>
+      <c r="D16" s="44"/>
       <c r="E16" s="5"/>
       <c r="F16" s="4"/>
-    </row>
-    <row r="17" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B17" s="32"/>
-      <c r="C17" s="39"/>
-      <c r="D17" s="33"/>
-      <c r="E17" s="10"/>
+      <c r="H16" s="15"/>
+      <c r="I16" s="49"/>
+      <c r="J16" s="49"/>
+      <c r="K16" s="49"/>
+      <c r="L16" s="49"/>
+      <c r="M16" s="49"/>
+      <c r="N16" s="49"/>
+      <c r="O16" s="49"/>
+      <c r="P16" s="49"/>
+      <c r="Q16" s="49"/>
+      <c r="R16" s="49"/>
+      <c r="S16" s="17"/>
+    </row>
+    <row r="17" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B17" s="42"/>
+      <c r="C17" s="43"/>
+      <c r="D17" s="44"/>
+      <c r="E17" s="8"/>
       <c r="F17" s="4"/>
-    </row>
-    <row r="19" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B19" s="37" t="s">
+      <c r="H17" s="15"/>
+      <c r="I17" s="49"/>
+      <c r="J17" s="49"/>
+      <c r="K17" s="49"/>
+      <c r="L17" s="49"/>
+      <c r="M17" s="49"/>
+      <c r="N17" s="49"/>
+      <c r="O17" s="49"/>
+      <c r="P17" s="49"/>
+      <c r="Q17" s="49"/>
+      <c r="R17" s="49"/>
+      <c r="S17" s="17"/>
+    </row>
+    <row r="18" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="H18" s="15"/>
+      <c r="I18" s="49"/>
+      <c r="J18" s="49"/>
+      <c r="K18" s="49"/>
+      <c r="L18" s="49"/>
+      <c r="M18" s="49"/>
+      <c r="N18" s="49"/>
+      <c r="O18" s="49"/>
+      <c r="P18" s="49"/>
+      <c r="Q18" s="49"/>
+      <c r="R18" s="49"/>
+      <c r="S18" s="17"/>
+    </row>
+    <row r="19" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B19" s="30" t="s">
         <v>53</v>
       </c>
-      <c r="C19" s="37"/>
-      <c r="D19" s="37"/>
-      <c r="E19" s="37"/>
-      <c r="F19" s="37"/>
-    </row>
-    <row r="20" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B20" s="37"/>
-      <c r="C20" s="37"/>
-      <c r="D20" s="37"/>
-      <c r="E20" s="37"/>
-      <c r="F20" s="37"/>
+      <c r="C19" s="30"/>
+      <c r="D19" s="30"/>
+      <c r="E19" s="30"/>
+      <c r="F19" s="30"/>
+      <c r="H19" s="15"/>
+      <c r="I19" s="49"/>
+      <c r="J19" s="49"/>
+      <c r="K19" s="49"/>
+      <c r="L19" s="49"/>
+      <c r="M19" s="49"/>
+      <c r="N19" s="49"/>
+      <c r="O19" s="49"/>
+      <c r="P19" s="49"/>
+      <c r="Q19" s="49"/>
+      <c r="R19" s="49"/>
+      <c r="S19" s="17"/>
+    </row>
+    <row r="20" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="B20" s="30"/>
+      <c r="C20" s="30"/>
+      <c r="D20" s="30"/>
+      <c r="E20" s="30"/>
+      <c r="F20" s="30"/>
+      <c r="H20" s="18"/>
+      <c r="I20" s="19"/>
+      <c r="J20" s="19"/>
+      <c r="K20" s="19"/>
+      <c r="L20" s="19"/>
+      <c r="M20" s="19"/>
+      <c r="N20" s="19"/>
+      <c r="O20" s="19"/>
+      <c r="P20" s="19"/>
+      <c r="Q20" s="19"/>
+      <c r="R20" s="19"/>
+      <c r="S20" s="20"/>
     </row>
   </sheetData>
   <mergeCells count="18">
-    <mergeCell ref="H15:J15"/>
+    <mergeCell ref="B19:F20"/>
+    <mergeCell ref="B11:D11"/>
+    <mergeCell ref="B16:D16"/>
+    <mergeCell ref="B17:D17"/>
+    <mergeCell ref="H9:I9"/>
+    <mergeCell ref="H12:S20"/>
     <mergeCell ref="B12:D15"/>
     <mergeCell ref="E12:E15"/>
     <mergeCell ref="F12:F15"/>
     <mergeCell ref="B2:O3"/>
     <mergeCell ref="H5:O5"/>
-    <mergeCell ref="B19:F20"/>
-    <mergeCell ref="B11:D11"/>
-    <mergeCell ref="B16:D16"/>
-    <mergeCell ref="B17:D17"/>
-    <mergeCell ref="H9:I9"/>
     <mergeCell ref="J6:K6"/>
     <mergeCell ref="J7:K7"/>
     <mergeCell ref="J8:K8"/>

</xml_diff>